<commit_message>
BDD day 1 commit
</commit_message>
<xml_diff>
--- a/Selenium/nykaa_end_to_end/test_data/data.xlsx
+++ b/Selenium/nykaa_end_to_end/test_data/data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/9598ef7ed350fd67/Documents/Yoga_5370346_WiproCapstone/Selenium/nykaa_end_to_end/test_data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="27" documentId="8_{28F531A5-0CD4-42AB-9789-D32F7E0F529A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E7248216-80B3-44FE-9DF8-7442C2684858}"/>
+  <xr:revisionPtr revIDLastSave="28" documentId="8_{28F531A5-0CD4-42AB-9789-D32F7E0F529A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{37B7D8ED-F78E-4597-9074-AE2432631044}"/>
   <bookViews>
-    <workbookView xWindow="380" yWindow="380" windowWidth="14400" windowHeight="7270" xr2:uid="{D404606D-13B5-4A31-A046-6C92B6895290}"/>
+    <workbookView minimized="1" xWindow="380" yWindow="380" windowWidth="14400" windowHeight="7270" xr2:uid="{D404606D-13B5-4A31-A046-6C92B6895290}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>

</xml_diff>